<commit_message>
Update state restriction crosswalk from revised PAP Table 1 and refresh outputs.
</commit_message>
<xml_diff>
--- a/output/tables/Table1_Descriptives.xlsx
+++ b/output/tables/Table1_Descriptives.xlsx
@@ -543,25 +543,25 @@
     <t xml:space="preserve">   Not adopted</t>
   </si>
   <si>
-    <t>4466 (51.2)</t>
-  </si>
-  <si>
-    <t>1915 (44.1)</t>
-  </si>
-  <si>
-    <t>2551 (58.3)</t>
+    <t>4454 (51.1)</t>
+  </si>
+  <si>
+    <t>1912 (44.1)</t>
+  </si>
+  <si>
+    <t>2542 (58.1)</t>
   </si>
   <si>
     <t xml:space="preserve">   Adopted not yet implemented or vacated</t>
   </si>
   <si>
-    <t>1060 (12.2)</t>
-  </si>
-  <si>
-    <t>523 (12.1)</t>
-  </si>
-  <si>
-    <t>537 (12.3)</t>
+    <t>1238 (14.2)</t>
+  </si>
+  <si>
+    <t>607 (14.0)</t>
+  </si>
+  <si>
+    <t>631 (14.4)</t>
   </si>
   <si>
     <t xml:space="preserve">   Previously implemented but vacated</t>
@@ -579,13 +579,13 @@
     <t xml:space="preserve">   Currently implemented</t>
   </si>
   <si>
-    <t>2866 (32.9)</t>
-  </si>
-  <si>
-    <t>1680 (38.7)</t>
-  </si>
-  <si>
-    <t>1186 (27.1)</t>
+    <t>2700 (31.0)</t>
+  </si>
+  <si>
+    <t>1599 (36.8)</t>
+  </si>
+  <si>
+    <t>1101 (25.2)</t>
   </si>
   <si>
     <t>Note. Complete-case analysis sample. Continuous variables reported as mean (SD); categorical covariates as n (% within column). Unweighted. Percentages may not sum to 100 because of rounding.</t>

</xml_diff>